<commit_message>
update NMA-for-EGFR-TKI v2.0 20250528
</commit_message>
<xml_diff>
--- a/NMA-for-EGFR-TKI/input/Forest plot subgroup.xlsx
+++ b/NMA-for-EGFR-TKI/input/Forest plot subgroup.xlsx
@@ -72,10 +72,10 @@
     <t>treat_line</t>
   </si>
   <si>
-    <t>front_line</t>
+    <t>first_line</t>
   </si>
   <si>
-    <t>front_line_chemo</t>
+    <t>first_line_chemo</t>
   </si>
   <si>
     <t>trial</t>

</xml_diff>